<commit_message>
Update logic for GEMINI
</commit_message>
<xml_diff>
--- a/data/May/THÁNG 5.2026- CHÂU NGÂN- ĐỐI SOÁT.xlsx
+++ b/data/May/THÁNG 5.2026- CHÂU NGÂN- ĐỐI SOÁT.xlsx
@@ -8,17 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\May\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{440E365E-38EF-4AAF-B041-E2C0A636220D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32148833-C6B8-40C6-9E96-9336EC4E3AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1-5" sheetId="3" r:id="rId1"/>
-    <sheet name="2-5" sheetId="4" r:id="rId2"/>
+    <sheet name="4-5" sheetId="4" r:id="rId2"/>
+    <sheet name="5-5" sheetId="5" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1-5'!$A$2:$P$56</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2-5'!$A$2:$P$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'4-5'!$A$2:$P$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'5-5'!$A$2:$P$56</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="269">
   <si>
     <t>Tình trạng TT</t>
   </si>
@@ -121,15 +123,6 @@
     <t>ĐỊA CHỈ</t>
   </si>
   <si>
-    <t>THU 7</t>
-  </si>
-  <si>
-    <t>NGAY 2-5</t>
-  </si>
-  <si>
-    <t>T7.2.5.2026</t>
-  </si>
-  <si>
     <t>THU 6</t>
   </si>
   <si>
@@ -662,6 +655,201 @@
   </si>
   <si>
     <t>135 hải thượng lãn ông P10</t>
+  </si>
+  <si>
+    <t>NGAY 4-5</t>
+  </si>
+  <si>
+    <t>THU 2</t>
+  </si>
+  <si>
+    <t>T2.4.5.2026</t>
+  </si>
+  <si>
+    <t>Hồ Thị Mỹ Hạnh</t>
+  </si>
+  <si>
+    <t>HD018199</t>
+  </si>
+  <si>
+    <t>S3.02 vinhomes garden park long bình</t>
+  </si>
+  <si>
+    <t>04-05-2026</t>
+  </si>
+  <si>
+    <t>Dạ Thảo (Hàng của Thanh đi Malaysia)</t>
+  </si>
+  <si>
+    <t>HD018104</t>
+  </si>
+  <si>
+    <t>66 đường số 17 phường 10</t>
+  </si>
+  <si>
+    <t>AT 04-05</t>
+  </si>
+  <si>
+    <t>hương</t>
+  </si>
+  <si>
+    <t>HD018201</t>
+  </si>
+  <si>
+    <t>97 đường 24A -bình trị đông b</t>
+  </si>
+  <si>
+    <t>Ngọc - fb Nguyễn Mười Ut</t>
+  </si>
+  <si>
+    <t>HD018123</t>
+  </si>
+  <si>
+    <t>45/8 đường số 8 phường bình hưng hòa A</t>
+  </si>
+  <si>
+    <t>Hạnh Huỳnh</t>
+  </si>
+  <si>
+    <t>HD018243</t>
+  </si>
+  <si>
+    <t>42A, đường Mã Lò, phường Bình Trị Đông A</t>
+  </si>
+  <si>
+    <t>Bé Bờm</t>
+  </si>
+  <si>
+    <t>HD018225</t>
+  </si>
+  <si>
+    <t>167/10 Đào Sư Tích, Phước Kiển</t>
+  </si>
+  <si>
+    <t>Quế Trân Nguyễn</t>
+  </si>
+  <si>
+    <t>HD018214</t>
+  </si>
+  <si>
+    <t>145 Nguyễn Cửu Đàm - Tân Sơn Nhì</t>
+  </si>
+  <si>
+    <t>Bé My</t>
+  </si>
+  <si>
+    <t>HD017792</t>
+  </si>
+  <si>
+    <t>304/45 đường số 8 bình hưng hoà a</t>
+  </si>
+  <si>
+    <t>chip chip</t>
+  </si>
+  <si>
+    <t>HD018274</t>
+  </si>
+  <si>
+    <t>71/16 thới an 16</t>
+  </si>
+  <si>
+    <t>My Nguyễn</t>
+  </si>
+  <si>
+    <t>HD018234</t>
+  </si>
+  <si>
+    <t>256/33 liên khu 4 - 5 - Bình Hưng Hòa B</t>
+  </si>
+  <si>
+    <t>Hoàng Trinh</t>
+  </si>
+  <si>
+    <t>HD018238</t>
+  </si>
+  <si>
+    <t>71/1/33.Nguyễn van Thuong p Thạnh mỹ tây</t>
+  </si>
+  <si>
+    <t>chi hương fb Kim Tien Phan</t>
+  </si>
+  <si>
+    <t>HD018239</t>
+  </si>
+  <si>
+    <t>328 đường số 8 thông tây hội</t>
+  </si>
+  <si>
+    <t>Kim Anh</t>
+  </si>
+  <si>
+    <t>HD018216</t>
+  </si>
+  <si>
+    <t>124/83/1 xô viết nghệ tĩnh p21</t>
+  </si>
+  <si>
+    <t>TRANG TRẦN 2</t>
+  </si>
+  <si>
+    <t>1122/23/7 quang trung phường 8</t>
+  </si>
+  <si>
+    <t>Qn Nguyễn</t>
+  </si>
+  <si>
+    <t>189/46a Bạch Đằng, phường Hạnh Thông</t>
+  </si>
+  <si>
+    <t>NIKI VIJANDRE + Air Shipment + Mien Tran</t>
+  </si>
+  <si>
+    <t>14 Lam Thi Ho, Tan Chanh Hiep Ward</t>
+  </si>
+  <si>
+    <t>Ngọc Thủy</t>
+  </si>
+  <si>
+    <t>41 Mạc Đĩnh Chi, đakao, P1</t>
+  </si>
+  <si>
+    <t>Mã Thục Phối</t>
+  </si>
+  <si>
+    <t>HD016561</t>
+  </si>
+  <si>
+    <t>156 hàn hải nguyên f8</t>
+  </si>
+  <si>
+    <t>Ngọc Tuyền</t>
+  </si>
+  <si>
+    <t>HD018193</t>
+  </si>
+  <si>
+    <t>Saigon Royal OT2</t>
+  </si>
+  <si>
+    <t>Người nhận chuột</t>
+  </si>
+  <si>
+    <t>HD018256</t>
+  </si>
+  <si>
+    <t>số 229A Đường bùi thị xuân phường 1</t>
+  </si>
+  <si>
+    <t>đơn trả 5.5</t>
+  </si>
+  <si>
+    <t>THU 3</t>
+  </si>
+  <si>
+    <t>NGAY 5-5</t>
+  </si>
+  <si>
+    <t>T3.5.5.2026</t>
   </si>
 </sst>
 </file>
@@ -1175,10 +1363,10 @@
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
@@ -1234,17 +1422,17 @@
     </row>
     <row r="3" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="22" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C3" s="22" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D3" s="22"/>
       <c r="E3" s="22" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F3" s="29">
         <v>9</v>
@@ -1260,13 +1448,13 @@
         <v>860</v>
       </c>
       <c r="J3" s="22" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="K3" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L3" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M3" s="22"/>
       <c r="N3" s="22"/>
@@ -1279,19 +1467,19 @@
     <row r="4" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="22"/>
       <c r="B4" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C4" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="29" t="s">
         <v>39</v>
-      </c>
-      <c r="D4" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="E4" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="F4" s="29" t="s">
-        <v>42</v>
       </c>
       <c r="G4" s="23">
         <v>920</v>
@@ -1304,13 +1492,13 @@
         <v>890</v>
       </c>
       <c r="J4" s="22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K4" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L4" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M4" s="22"/>
       <c r="N4" s="22"/>
@@ -1323,16 +1511,16 @@
     <row r="5" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="22"/>
       <c r="B5" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E5" s="22" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F5" s="29">
         <v>12</v>
@@ -1348,13 +1536,13 @@
         <v>860</v>
       </c>
       <c r="J5" s="22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K5" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L5" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M5" s="22"/>
       <c r="N5" s="22"/>
@@ -1367,16 +1555,16 @@
     <row r="6" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="22"/>
       <c r="B6" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C6" s="22" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F6" s="29">
         <v>12</v>
@@ -1392,13 +1580,13 @@
         <v>350</v>
       </c>
       <c r="J6" s="22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K6" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L6" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M6" s="22"/>
       <c r="N6" s="22"/>
@@ -1411,16 +1599,16 @@
     <row r="7" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="22"/>
       <c r="B7" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F7" s="29">
         <v>8</v>
@@ -1436,13 +1624,13 @@
         <v>470</v>
       </c>
       <c r="J7" s="22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K7" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L7" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M7" s="22"/>
       <c r="N7" s="22"/>
@@ -1455,16 +1643,16 @@
     <row r="8" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="22"/>
       <c r="B8" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F8" s="29">
         <v>8</v>
@@ -1480,13 +1668,13 @@
         <v>860</v>
       </c>
       <c r="J8" s="22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K8" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L8" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M8" s="22"/>
       <c r="N8" s="22"/>
@@ -1499,16 +1687,16 @@
     <row r="9" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="22"/>
       <c r="B9" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F9" s="29">
         <v>12</v>
@@ -1524,13 +1712,13 @@
         <v>-30</v>
       </c>
       <c r="J9" s="22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K9" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L9" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M9" s="22"/>
       <c r="N9" s="22"/>
@@ -1547,19 +1735,19 @@
     <row r="10" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="22"/>
       <c r="B10" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C10" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="F10" s="29" t="s">
         <v>59</v>
-      </c>
-      <c r="D10" s="22" t="s">
-        <v>60</v>
-      </c>
-      <c r="E10" s="22" t="s">
-        <v>61</v>
-      </c>
-      <c r="F10" s="29" t="s">
-        <v>62</v>
       </c>
       <c r="G10" s="23">
         <v>785</v>
@@ -1572,13 +1760,13 @@
         <v>760</v>
       </c>
       <c r="J10" s="22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K10" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L10" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M10" s="22"/>
       <c r="N10" s="22"/>
@@ -1591,19 +1779,19 @@
     <row r="11" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="22"/>
       <c r="B11" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D11" s="22" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E11" s="22" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F11" s="29" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G11" s="23">
         <v>720</v>
@@ -1616,13 +1804,13 @@
         <v>690</v>
       </c>
       <c r="J11" s="22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K11" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L11" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M11" s="22"/>
       <c r="N11" s="22"/>
@@ -1635,16 +1823,16 @@
     <row r="12" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="22"/>
       <c r="B12" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D12" s="22" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F12" s="29">
         <v>8</v>
@@ -1660,13 +1848,13 @@
         <v>750</v>
       </c>
       <c r="J12" s="22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K12" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L12" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M12" s="22"/>
       <c r="N12" s="22"/>
@@ -1679,19 +1867,19 @@
     <row r="13" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="22"/>
       <c r="B13" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C13" s="22" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D13" s="22" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F13" s="29" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G13" s="23">
         <v>670</v>
@@ -1704,13 +1892,13 @@
         <v>640</v>
       </c>
       <c r="J13" s="22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K13" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L13" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M13" s="22"/>
       <c r="N13" s="22"/>
@@ -1723,16 +1911,16 @@
     <row r="14" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="22"/>
       <c r="B14" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D14" s="22" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E14" s="22" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F14" s="29">
         <v>6</v>
@@ -1748,13 +1936,13 @@
         <v>1420</v>
       </c>
       <c r="J14" s="22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K14" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L14" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M14" s="22"/>
       <c r="N14" s="22"/>
@@ -1767,16 +1955,16 @@
     <row r="15" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="22"/>
       <c r="B15" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C15" s="22" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F15" s="29">
         <v>9</v>
@@ -1792,13 +1980,13 @@
         <v>750</v>
       </c>
       <c r="J15" s="22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K15" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L15" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M15" s="22"/>
       <c r="N15" s="22"/>
@@ -1811,19 +1999,19 @@
     <row r="16" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="22"/>
       <c r="B16" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D16" s="22" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F16" s="29" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G16" s="23">
         <v>0</v>
@@ -1836,13 +2024,13 @@
         <v>-30</v>
       </c>
       <c r="J16" s="22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K16" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L16" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M16" s="22"/>
       <c r="N16" s="22"/>
@@ -1859,16 +2047,16 @@
     <row r="17" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="22"/>
       <c r="B17" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D17" s="22" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F17" s="29">
         <v>12</v>
@@ -1884,13 +2072,13 @@
         <v>660</v>
       </c>
       <c r="J17" s="22" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="K17" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L17" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M17" s="22"/>
       <c r="N17" s="22"/>
@@ -1903,16 +2091,16 @@
     <row r="18" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="22"/>
       <c r="B18" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D18" s="22" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="E18" s="22" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="F18" s="29">
         <v>2</v>
@@ -1928,13 +2116,13 @@
         <v>790</v>
       </c>
       <c r="J18" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K18" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L18" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M18" s="22"/>
       <c r="N18" s="22"/>
@@ -1947,16 +2135,16 @@
     <row r="19" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="22"/>
       <c r="B19" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E19" s="22" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="F19" s="29">
         <v>12</v>
@@ -1972,13 +2160,13 @@
         <v>-30</v>
       </c>
       <c r="J19" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K19" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L19" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M19" s="22"/>
       <c r="N19" s="22"/>
@@ -1995,19 +2183,19 @@
     <row r="20" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="22"/>
       <c r="B20" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C20" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="D20" s="22" t="s">
+        <v>88</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F20" s="29" t="s">
         <v>90</v>
-      </c>
-      <c r="D20" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="E20" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="F20" s="29" t="s">
-        <v>93</v>
       </c>
       <c r="G20" s="23">
         <v>0</v>
@@ -2020,13 +2208,13 @@
         <v>-40</v>
       </c>
       <c r="J20" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K20" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L20" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M20" s="22"/>
       <c r="N20" s="22"/>
@@ -2043,19 +2231,19 @@
     <row r="21" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="22"/>
       <c r="B21" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C21" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="D21" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="E21" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="F21" s="29" t="s">
         <v>94</v>
-      </c>
-      <c r="D21" s="22" t="s">
-        <v>95</v>
-      </c>
-      <c r="E21" s="22" t="s">
-        <v>96</v>
-      </c>
-      <c r="F21" s="29" t="s">
-        <v>97</v>
       </c>
       <c r="G21" s="23">
         <v>690</v>
@@ -2068,13 +2256,13 @@
         <v>660</v>
       </c>
       <c r="J21" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K21" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L21" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M21" s="22"/>
       <c r="N21" s="22"/>
@@ -2087,19 +2275,19 @@
     <row r="22" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="22"/>
       <c r="B22" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C22" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="D22" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="E22" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="F22" s="29" t="s">
         <v>98</v>
-      </c>
-      <c r="D22" s="22" t="s">
-        <v>99</v>
-      </c>
-      <c r="E22" s="22" t="s">
-        <v>100</v>
-      </c>
-      <c r="F22" s="29" t="s">
-        <v>101</v>
       </c>
       <c r="G22" s="23">
         <v>660</v>
@@ -2112,13 +2300,13 @@
         <v>640</v>
       </c>
       <c r="J22" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K22" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L22" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M22" s="22"/>
       <c r="N22" s="22"/>
@@ -2131,19 +2319,19 @@
     <row r="23" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="22"/>
       <c r="B23" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D23" s="22" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="F23" s="29" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G23" s="23">
         <v>375</v>
@@ -2156,13 +2344,13 @@
         <v>350</v>
       </c>
       <c r="J23" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K23" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L23" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M23" s="22"/>
       <c r="N23" s="22"/>
@@ -2175,19 +2363,19 @@
     <row r="24" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="22"/>
       <c r="B24" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C24" s="22" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D24" s="22" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E24" s="22" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="F24" s="29" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G24" s="23">
         <v>0</v>
@@ -2200,13 +2388,13 @@
         <v>-25</v>
       </c>
       <c r="J24" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K24" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L24" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M24" s="22"/>
       <c r="N24" s="22"/>
@@ -2223,19 +2411,19 @@
     <row r="25" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="22"/>
       <c r="B25" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C25" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="D25" s="22" t="s">
+        <v>106</v>
+      </c>
+      <c r="E25" s="22" t="s">
+        <v>107</v>
+      </c>
+      <c r="F25" s="29" t="s">
         <v>108</v>
-      </c>
-      <c r="D25" s="22" t="s">
-        <v>109</v>
-      </c>
-      <c r="E25" s="22" t="s">
-        <v>110</v>
-      </c>
-      <c r="F25" s="29" t="s">
-        <v>111</v>
       </c>
       <c r="G25" s="23">
         <v>725</v>
@@ -2248,13 +2436,13 @@
         <v>700</v>
       </c>
       <c r="J25" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K25" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L25" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M25" s="22"/>
       <c r="N25" s="22"/>
@@ -2267,19 +2455,19 @@
     <row r="26" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="22"/>
       <c r="B26" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C26" s="22" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D26" s="22" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E26" s="22" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="F26" s="29" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G26" s="23">
         <v>0</v>
@@ -2292,13 +2480,13 @@
         <v>-25</v>
       </c>
       <c r="J26" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K26" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L26" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M26" s="22"/>
       <c r="N26" s="22"/>
@@ -2315,19 +2503,19 @@
     <row r="27" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="22"/>
       <c r="B27" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C27" s="22" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D27" s="22" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="E27" s="22" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="F27" s="29" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G27" s="23">
         <v>1765</v>
@@ -2340,13 +2528,13 @@
         <v>1740</v>
       </c>
       <c r="J27" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K27" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L27" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M27" s="22"/>
       <c r="N27" s="22"/>
@@ -2359,19 +2547,19 @@
     <row r="28" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="22"/>
       <c r="B28" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C28" s="22" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D28" s="22" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E28" s="22" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="F28" s="29" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G28" s="23">
         <v>0</v>
@@ -2384,13 +2572,13 @@
         <v>-25</v>
       </c>
       <c r="J28" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K28" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L28" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M28" s="22"/>
       <c r="N28" s="22"/>
@@ -2407,19 +2595,19 @@
     <row r="29" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="22"/>
       <c r="B29" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C29" s="22" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D29" s="22" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="F29" s="29" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G29" s="23">
         <v>765</v>
@@ -2432,13 +2620,13 @@
         <v>740</v>
       </c>
       <c r="J29" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K29" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L29" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M29" s="22"/>
       <c r="N29" s="22"/>
@@ -2451,19 +2639,19 @@
     <row r="30" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="22"/>
       <c r="B30" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D30" s="22" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="E30" s="22" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="F30" s="29" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="G30" s="23">
         <v>820</v>
@@ -2476,13 +2664,13 @@
         <v>790</v>
       </c>
       <c r="J30" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K30" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L30" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M30" s="22"/>
       <c r="N30" s="22"/>
@@ -2495,19 +2683,19 @@
     <row r="31" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="22"/>
       <c r="B31" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D31" s="22" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="F31" s="29" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="G31" s="23">
         <v>740</v>
@@ -2520,13 +2708,13 @@
         <v>720</v>
       </c>
       <c r="J31" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K31" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L31" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M31" s="22"/>
       <c r="N31" s="22"/>
@@ -2539,19 +2727,19 @@
     <row r="32" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="22"/>
       <c r="B32" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C32" s="22" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D32" s="22" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E32" s="22" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F32" s="29" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="G32" s="23">
         <v>770</v>
@@ -2564,13 +2752,13 @@
         <v>750</v>
       </c>
       <c r="J32" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K32" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L32" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M32" s="22"/>
       <c r="N32" s="22"/>
@@ -2583,16 +2771,16 @@
     <row r="33" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="22"/>
       <c r="B33" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C33" s="22" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D33" s="22" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E33" s="22" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F33" s="29">
         <v>2</v>
@@ -2608,13 +2796,13 @@
         <v>-30</v>
       </c>
       <c r="J33" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K33" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L33" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M33" s="22"/>
       <c r="N33" s="22"/>
@@ -2631,19 +2819,19 @@
     <row r="34" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="22"/>
       <c r="B34" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D34" s="22" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="E34" s="22" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="F34" s="29" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="G34" s="23">
         <v>590</v>
@@ -2656,13 +2844,13 @@
         <v>570</v>
       </c>
       <c r="J34" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K34" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L34" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M34" s="22"/>
       <c r="N34" s="22"/>
@@ -2675,16 +2863,16 @@
     <row r="35" spans="1:18" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="25"/>
       <c r="B35" s="25" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C35" s="25" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D35" s="25" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E35" s="25" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F35" s="30">
         <v>2</v>
@@ -2700,16 +2888,16 @@
         <v>80</v>
       </c>
       <c r="J35" s="25" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K35" s="25" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L35" s="25" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M35" s="25" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="N35" s="25"/>
       <c r="O35" s="25"/>
@@ -2720,20 +2908,20 @@
     </row>
     <row r="36" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="22" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B36" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D36" s="22"/>
       <c r="E36" s="22" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F36" s="29" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="G36" s="23">
         <v>1165</v>
@@ -2746,13 +2934,13 @@
         <v>1130</v>
       </c>
       <c r="J36" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K36" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L36" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M36" s="22"/>
       <c r="N36" s="22"/>
@@ -2764,20 +2952,20 @@
     </row>
     <row r="37" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="22" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B37" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D37" s="22"/>
       <c r="E37" s="22" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F37" s="29" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G37" s="23">
         <v>2985</v>
@@ -2790,13 +2978,13 @@
         <v>2950</v>
       </c>
       <c r="J37" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K37" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L37" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M37" s="22"/>
       <c r="N37" s="22"/>
@@ -2809,19 +2997,19 @@
     <row r="38" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="22"/>
       <c r="B38" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C38" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="D38" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="E38" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="F38" s="29" t="s">
         <v>147</v>
-      </c>
-      <c r="D38" s="22" t="s">
-        <v>148</v>
-      </c>
-      <c r="E38" s="22" t="s">
-        <v>149</v>
-      </c>
-      <c r="F38" s="29" t="s">
-        <v>150</v>
       </c>
       <c r="G38" s="23">
         <v>1145</v>
@@ -2834,13 +3022,13 @@
         <v>1110</v>
       </c>
       <c r="J38" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K38" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L38" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M38" s="22"/>
       <c r="N38" s="22"/>
@@ -2853,19 +3041,19 @@
     <row r="39" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="22"/>
       <c r="B39" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C39" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="D39" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="E39" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="F39" s="29" t="s">
         <v>152</v>
-      </c>
-      <c r="D39" s="22" t="s">
-        <v>153</v>
-      </c>
-      <c r="E39" s="22" t="s">
-        <v>154</v>
-      </c>
-      <c r="F39" s="29" t="s">
-        <v>155</v>
       </c>
       <c r="G39" s="23">
         <v>675</v>
@@ -2878,13 +3066,13 @@
         <v>640</v>
       </c>
       <c r="J39" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K39" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L39" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M39" s="22"/>
       <c r="N39" s="22"/>
@@ -2897,16 +3085,16 @@
     <row r="40" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="22"/>
       <c r="B40" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C40" s="22" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D40" s="22" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="E40" s="22" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="F40" s="29">
         <v>5</v>
@@ -2922,13 +3110,13 @@
         <v>760</v>
       </c>
       <c r="J40" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K40" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L40" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M40" s="22"/>
       <c r="N40" s="22"/>
@@ -2941,16 +3129,16 @@
     <row r="41" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="22"/>
       <c r="B41" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C41" s="22" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D41" s="22" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E41" s="22" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="F41" s="29">
         <v>1</v>
@@ -2966,13 +3154,13 @@
         <v>700</v>
       </c>
       <c r="J41" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K41" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L41" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M41" s="22"/>
       <c r="N41" s="22"/>
@@ -2985,16 +3173,16 @@
     <row r="42" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="22"/>
       <c r="B42" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D42" s="22" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="E42" s="22" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F42" s="29">
         <v>5</v>
@@ -3010,13 +3198,13 @@
         <v>-25</v>
       </c>
       <c r="J42" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K42" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L42" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M42" s="22"/>
       <c r="N42" s="22"/>
@@ -3033,16 +3221,16 @@
     <row r="43" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="22"/>
       <c r="B43" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D43" s="22" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="E43" s="22" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F43" s="29">
         <v>3</v>
@@ -3058,13 +3246,13 @@
         <v>1560</v>
       </c>
       <c r="J43" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K43" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L43" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M43" s="22"/>
       <c r="N43" s="22"/>
@@ -3077,16 +3265,16 @@
     <row r="44" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="22"/>
       <c r="B44" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="D44" s="22" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E44" s="22" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="F44" s="29">
         <v>3</v>
@@ -3102,13 +3290,13 @@
         <v>790</v>
       </c>
       <c r="J44" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K44" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L44" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M44" s="22"/>
       <c r="N44" s="22"/>
@@ -3121,16 +3309,16 @@
     <row r="45" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="22"/>
       <c r="B45" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C45" s="22" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D45" s="22" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="E45" s="22" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F45" s="29">
         <v>7</v>
@@ -3146,13 +3334,13 @@
         <v>660</v>
       </c>
       <c r="J45" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K45" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L45" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M45" s="22"/>
       <c r="N45" s="22"/>
@@ -3165,19 +3353,19 @@
     <row r="46" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="22"/>
       <c r="B46" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C46" s="22" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D46" s="22" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="E46" s="22" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="F46" s="29" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="G46" s="23">
         <v>0</v>
@@ -3190,13 +3378,13 @@
         <v>-25</v>
       </c>
       <c r="J46" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K46" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L46" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M46" s="22"/>
       <c r="N46" s="22"/>
@@ -3210,63 +3398,65 @@
         <v>25</v>
       </c>
     </row>
-    <row r="47" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="22"/>
-      <c r="B47" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="C47" s="22" t="s">
-        <v>177</v>
-      </c>
-      <c r="D47" s="22" t="s">
-        <v>178</v>
-      </c>
-      <c r="E47" s="22" t="s">
-        <v>179</v>
-      </c>
-      <c r="F47" s="29">
+    <row r="47" spans="1:18" s="27" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="25"/>
+      <c r="B47" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="C47" s="25" t="s">
+        <v>174</v>
+      </c>
+      <c r="D47" s="25" t="s">
+        <v>175</v>
+      </c>
+      <c r="E47" s="25" t="s">
+        <v>176</v>
+      </c>
+      <c r="F47" s="30">
         <v>7</v>
       </c>
-      <c r="G47" s="23">
-        <v>720</v>
-      </c>
-      <c r="H47" s="23">
-        <v>30</v>
-      </c>
-      <c r="I47" s="23">
+      <c r="G47" s="26">
+        <v>60</v>
+      </c>
+      <c r="H47" s="26">
+        <v>30</v>
+      </c>
+      <c r="I47" s="26">
         <f>G47-H47</f>
-        <v>690</v>
-      </c>
-      <c r="J47" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="K47" s="22" t="s">
-        <v>37</v>
-      </c>
-      <c r="L47" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="M47" s="22"/>
-      <c r="N47" s="22"/>
-      <c r="O47" s="22"/>
-      <c r="P47" s="22"/>
-      <c r="Q47" s="22">
+        <v>30</v>
+      </c>
+      <c r="J47" s="25" t="s">
+        <v>148</v>
+      </c>
+      <c r="K47" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="L47" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="M47" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="N47" s="25"/>
+      <c r="O47" s="25"/>
+      <c r="P47" s="25"/>
+      <c r="Q47" s="25">
         <v>1</v>
       </c>
     </row>
     <row r="48" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="22"/>
       <c r="B48" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C48" s="22" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D48" s="22" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="E48" s="22" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="F48" s="29">
         <v>1</v>
@@ -3282,16 +3472,16 @@
         <v>2010</v>
       </c>
       <c r="J48" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K48" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L48" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M48" s="28" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="N48" s="22"/>
       <c r="O48" s="22"/>
@@ -3307,16 +3497,16 @@
     <row r="49" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="22"/>
       <c r="B49" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C49" s="22" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="D49" s="22" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="E49" s="22" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="F49" s="29">
         <v>7</v>
@@ -3332,13 +3522,13 @@
         <v>1770</v>
       </c>
       <c r="J49" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K49" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L49" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M49" s="22"/>
       <c r="N49" s="22"/>
@@ -3351,16 +3541,16 @@
     <row r="50" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="22"/>
       <c r="B50" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C50" s="22" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D50" s="22" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="E50" s="22" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="F50" s="29">
         <v>7</v>
@@ -3376,13 +3566,13 @@
         <v>740</v>
       </c>
       <c r="J50" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K50" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L50" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M50" s="22"/>
       <c r="N50" s="22"/>
@@ -3395,16 +3585,16 @@
     <row r="51" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="22"/>
       <c r="B51" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C51" s="22" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="D51" s="22" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="E51" s="22" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="F51" s="29">
         <v>7</v>
@@ -3420,13 +3610,13 @@
         <v>740</v>
       </c>
       <c r="J51" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K51" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L51" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M51" s="22"/>
       <c r="N51" s="22"/>
@@ -3439,16 +3629,16 @@
     <row r="52" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="22"/>
       <c r="B52" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C52" s="22" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D52" s="22" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="E52" s="22" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="F52" s="29">
         <v>8</v>
@@ -3464,13 +3654,13 @@
         <v>-25</v>
       </c>
       <c r="J52" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K52" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L52" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M52" s="22"/>
       <c r="N52" s="22"/>
@@ -3487,16 +3677,16 @@
     <row r="53" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="22"/>
       <c r="B53" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C53" s="22" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D53" s="22" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E53" s="22" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="F53" s="29">
         <v>3</v>
@@ -3512,13 +3702,13 @@
         <v>-25</v>
       </c>
       <c r="J53" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K53" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L53" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M53" s="22"/>
       <c r="N53" s="22"/>
@@ -3535,16 +3725,16 @@
     <row r="54" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="22"/>
       <c r="B54" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C54" s="22" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D54" s="22" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="E54" s="22" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="F54" s="29">
         <v>4</v>
@@ -3560,13 +3750,13 @@
         <v>790</v>
       </c>
       <c r="J54" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K54" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L54" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M54" s="22"/>
       <c r="N54" s="22"/>
@@ -3579,16 +3769,16 @@
     <row r="55" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="22"/>
       <c r="B55" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C55" s="22" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D55" s="22" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="E55" s="22" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="F55" s="29">
         <v>4</v>
@@ -3604,13 +3794,13 @@
         <v>790</v>
       </c>
       <c r="J55" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K55" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L55" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M55" s="22"/>
       <c r="N55" s="22"/>
@@ -3622,17 +3812,17 @@
     </row>
     <row r="56" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="22" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B56" s="22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C56" s="22" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="D56" s="22"/>
       <c r="E56" s="22" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F56" s="29">
         <v>5</v>
@@ -3648,13 +3838,13 @@
         <v>-30</v>
       </c>
       <c r="J56" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K56" s="22" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="L56" s="22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="M56" s="22"/>
       <c r="N56" s="22"/>
@@ -3671,7 +3861,7 @@
     <row r="58" spans="1:18" x14ac:dyDescent="0.25">
       <c r="G58" s="1">
         <f t="shared" ref="G58:R58" si="5">SUBTOTAL(9,G3:G57)</f>
-        <v>37475</v>
+        <v>36815</v>
       </c>
       <c r="H58" s="1">
         <f t="shared" si="5"/>
@@ -3679,7 +3869,7 @@
       </c>
       <c r="I58" s="1">
         <f t="shared" si="5"/>
-        <v>35955</v>
+        <v>35295</v>
       </c>
       <c r="J58" s="1">
         <f t="shared" si="5"/>
@@ -3720,7 +3910,7 @@
     </row>
     <row r="62" spans="1:18" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H62" s="4" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="I62" s="5" t="s">
         <v>15</v>
@@ -3735,7 +3925,7 @@
       </c>
       <c r="I63" s="8">
         <f>SUM(I57:I61)</f>
-        <v>35955</v>
+        <v>35295</v>
       </c>
       <c r="J63" s="8">
         <f>Q58</f>
@@ -3802,7 +3992,7 @@
       </c>
       <c r="I70" s="16">
         <f>SUM(I63:I69)</f>
-        <v>36350</v>
+        <v>35690</v>
       </c>
       <c r="J70" s="16">
         <f>SUM(J63:J67)</f>
@@ -3822,6 +4012,1129 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC23166D-647F-4247-A049-709567A97092}">
+  <dimension ref="A1:R36"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="9.140625" style="1"/>
+    <col min="3" max="3" width="27.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="67" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="11" width="9.140625" style="1"/>
+    <col min="12" max="12" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.42578125" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q2" s="3"/>
+    </row>
+    <row r="3" spans="1:17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="22"/>
+      <c r="B3" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>207</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>208</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>209</v>
+      </c>
+      <c r="F3" s="23">
+        <v>9</v>
+      </c>
+      <c r="G3" s="23">
+        <v>60</v>
+      </c>
+      <c r="H3" s="23">
+        <v>30</v>
+      </c>
+      <c r="I3" s="23">
+        <f>G3-H3</f>
+        <v>30</v>
+      </c>
+      <c r="J3" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="K3" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L3" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M3" s="22" t="s">
+        <v>180</v>
+      </c>
+      <c r="N3" s="22"/>
+      <c r="O3" s="22"/>
+      <c r="P3" s="22"/>
+      <c r="Q3" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="22"/>
+      <c r="B4" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>211</v>
+      </c>
+      <c r="D4" s="22" t="s">
+        <v>212</v>
+      </c>
+      <c r="E4" s="22" t="s">
+        <v>213</v>
+      </c>
+      <c r="F4" s="23">
+        <v>6</v>
+      </c>
+      <c r="G4" s="23">
+        <v>0</v>
+      </c>
+      <c r="H4" s="23">
+        <v>25</v>
+      </c>
+      <c r="I4" s="23">
+        <f>-H4</f>
+        <v>-25</v>
+      </c>
+      <c r="J4" s="22" t="s">
+        <v>214</v>
+      </c>
+      <c r="K4" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="22"/>
+      <c r="P4" s="22"/>
+      <c r="Q4" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="22"/>
+      <c r="B5" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>215</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>216</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>217</v>
+      </c>
+      <c r="F5" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="G5" s="23">
+        <v>0</v>
+      </c>
+      <c r="H5" s="23">
+        <v>30</v>
+      </c>
+      <c r="I5" s="23">
+        <f>-H5</f>
+        <v>-30</v>
+      </c>
+      <c r="J5" s="22" t="s">
+        <v>214</v>
+      </c>
+      <c r="K5" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M5" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="N5" s="22"/>
+      <c r="O5" s="22"/>
+      <c r="P5" s="22"/>
+      <c r="Q5" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="22"/>
+      <c r="B6" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>218</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>219</v>
+      </c>
+      <c r="E6" s="22" t="s">
+        <v>220</v>
+      </c>
+      <c r="F6" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" s="23">
+        <v>0</v>
+      </c>
+      <c r="H6" s="23">
+        <v>30</v>
+      </c>
+      <c r="I6" s="23">
+        <f>-H6</f>
+        <v>-30</v>
+      </c>
+      <c r="J6" s="22" t="s">
+        <v>214</v>
+      </c>
+      <c r="K6" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M6" s="22"/>
+      <c r="N6" s="22"/>
+      <c r="O6" s="22"/>
+      <c r="P6" s="22"/>
+      <c r="Q6" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="22"/>
+      <c r="B7" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>221</v>
+      </c>
+      <c r="D7" s="22" t="s">
+        <v>222</v>
+      </c>
+      <c r="E7" s="22" t="s">
+        <v>223</v>
+      </c>
+      <c r="F7" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="G7" s="23">
+        <v>820</v>
+      </c>
+      <c r="H7" s="23">
+        <v>30</v>
+      </c>
+      <c r="I7" s="23">
+        <f t="shared" ref="I7:I12" si="0">G7-H7</f>
+        <v>790</v>
+      </c>
+      <c r="J7" s="22" t="s">
+        <v>214</v>
+      </c>
+      <c r="K7" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L7" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M7" s="22"/>
+      <c r="N7" s="22"/>
+      <c r="O7" s="22"/>
+      <c r="P7" s="22"/>
+      <c r="Q7" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="22"/>
+      <c r="B8" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>224</v>
+      </c>
+      <c r="D8" s="22" t="s">
+        <v>225</v>
+      </c>
+      <c r="E8" s="22" t="s">
+        <v>226</v>
+      </c>
+      <c r="F8" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="G8" s="23">
+        <v>35</v>
+      </c>
+      <c r="H8" s="23">
+        <v>35</v>
+      </c>
+      <c r="I8" s="23">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J8" s="22" t="s">
+        <v>214</v>
+      </c>
+      <c r="K8" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L8" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M8" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="N8" s="22"/>
+      <c r="O8" s="22"/>
+      <c r="P8" s="22"/>
+      <c r="Q8" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="22"/>
+      <c r="B9" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>227</v>
+      </c>
+      <c r="D9" s="22" t="s">
+        <v>228</v>
+      </c>
+      <c r="E9" s="22" t="s">
+        <v>229</v>
+      </c>
+      <c r="F9" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="G9" s="23">
+        <v>985</v>
+      </c>
+      <c r="H9" s="23">
+        <v>25</v>
+      </c>
+      <c r="I9" s="23">
+        <f t="shared" si="0"/>
+        <v>960</v>
+      </c>
+      <c r="J9" s="22" t="s">
+        <v>214</v>
+      </c>
+      <c r="K9" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L9" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M9" s="22"/>
+      <c r="N9" s="22"/>
+      <c r="O9" s="22"/>
+      <c r="P9" s="22"/>
+      <c r="Q9" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="22"/>
+      <c r="B10" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>230</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>231</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>232</v>
+      </c>
+      <c r="F10" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="G10" s="23">
+        <v>1430</v>
+      </c>
+      <c r="H10" s="23">
+        <v>30</v>
+      </c>
+      <c r="I10" s="23">
+        <f t="shared" si="0"/>
+        <v>1400</v>
+      </c>
+      <c r="J10" s="22" t="s">
+        <v>214</v>
+      </c>
+      <c r="K10" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L10" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M10" s="22"/>
+      <c r="N10" s="22"/>
+      <c r="O10" s="22"/>
+      <c r="P10" s="22"/>
+      <c r="Q10" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="22"/>
+      <c r="B11" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>233</v>
+      </c>
+      <c r="D11" s="22" t="s">
+        <v>234</v>
+      </c>
+      <c r="E11" s="22" t="s">
+        <v>235</v>
+      </c>
+      <c r="F11" s="23">
+        <v>12</v>
+      </c>
+      <c r="G11" s="23">
+        <v>890</v>
+      </c>
+      <c r="H11" s="23">
+        <v>30</v>
+      </c>
+      <c r="I11" s="23">
+        <f t="shared" si="0"/>
+        <v>860</v>
+      </c>
+      <c r="J11" s="22" t="s">
+        <v>214</v>
+      </c>
+      <c r="K11" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L11" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M11" s="22"/>
+      <c r="N11" s="22"/>
+      <c r="O11" s="22"/>
+      <c r="P11" s="22"/>
+      <c r="Q11" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="22"/>
+      <c r="B12" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>236</v>
+      </c>
+      <c r="D12" s="22" t="s">
+        <v>237</v>
+      </c>
+      <c r="E12" s="22" t="s">
+        <v>238</v>
+      </c>
+      <c r="F12" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="G12" s="23">
+        <v>770</v>
+      </c>
+      <c r="H12" s="23">
+        <v>30</v>
+      </c>
+      <c r="I12" s="23">
+        <f t="shared" si="0"/>
+        <v>740</v>
+      </c>
+      <c r="J12" s="22" t="s">
+        <v>214</v>
+      </c>
+      <c r="K12" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L12" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M12" s="22"/>
+      <c r="N12" s="22"/>
+      <c r="O12" s="22"/>
+      <c r="P12" s="22"/>
+      <c r="Q12" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="22"/>
+      <c r="B13" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>239</v>
+      </c>
+      <c r="D13" s="22" t="s">
+        <v>240</v>
+      </c>
+      <c r="E13" s="22" t="s">
+        <v>241</v>
+      </c>
+      <c r="F13" s="22" t="s">
+        <v>98</v>
+      </c>
+      <c r="G13" s="23">
+        <v>0</v>
+      </c>
+      <c r="H13" s="23">
+        <v>20</v>
+      </c>
+      <c r="I13" s="23">
+        <f>-H13</f>
+        <v>-20</v>
+      </c>
+      <c r="J13" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="K13" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L13" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M13" s="22"/>
+      <c r="N13" s="22"/>
+      <c r="O13" s="22"/>
+      <c r="P13" s="22"/>
+      <c r="Q13" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="22"/>
+      <c r="B14" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>242</v>
+      </c>
+      <c r="D14" s="22" t="s">
+        <v>243</v>
+      </c>
+      <c r="E14" s="22" t="s">
+        <v>244</v>
+      </c>
+      <c r="F14" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="G14" s="23">
+        <v>905</v>
+      </c>
+      <c r="H14" s="23">
+        <v>25</v>
+      </c>
+      <c r="I14" s="23">
+        <f>G14-H14</f>
+        <v>880</v>
+      </c>
+      <c r="J14" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="K14" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L14" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M14" s="22"/>
+      <c r="N14" s="22"/>
+      <c r="O14" s="22"/>
+      <c r="P14" s="22"/>
+      <c r="Q14" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="22"/>
+      <c r="B15" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>245</v>
+      </c>
+      <c r="D15" s="22" t="s">
+        <v>246</v>
+      </c>
+      <c r="E15" s="22" t="s">
+        <v>247</v>
+      </c>
+      <c r="F15" s="22" t="s">
+        <v>98</v>
+      </c>
+      <c r="G15" s="23">
+        <v>0</v>
+      </c>
+      <c r="H15" s="23">
+        <v>20</v>
+      </c>
+      <c r="I15" s="23">
+        <f>-H15</f>
+        <v>-20</v>
+      </c>
+      <c r="J15" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="K15" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L15" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M15" s="22"/>
+      <c r="N15" s="22"/>
+      <c r="O15" s="22"/>
+      <c r="P15" s="22"/>
+      <c r="Q15" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>248</v>
+      </c>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22" t="s">
+        <v>249</v>
+      </c>
+      <c r="F16" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="G16" s="23">
+        <v>0</v>
+      </c>
+      <c r="H16" s="23">
+        <v>40</v>
+      </c>
+      <c r="I16" s="23">
+        <f>-H16</f>
+        <v>-40</v>
+      </c>
+      <c r="J16" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="K16" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L16" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M16" s="22"/>
+      <c r="N16" s="22"/>
+      <c r="O16" s="22"/>
+      <c r="P16" s="22"/>
+      <c r="Q16" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>250</v>
+      </c>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22" t="s">
+        <v>251</v>
+      </c>
+      <c r="F17" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="G17" s="23">
+        <v>1720</v>
+      </c>
+      <c r="H17" s="23">
+        <v>30</v>
+      </c>
+      <c r="I17" s="23">
+        <f>G17-H17</f>
+        <v>1690</v>
+      </c>
+      <c r="J17" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="K17" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L17" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M17" s="22"/>
+      <c r="N17" s="22"/>
+      <c r="O17" s="22"/>
+      <c r="P17" s="22"/>
+      <c r="Q17" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>252</v>
+      </c>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22" t="s">
+        <v>253</v>
+      </c>
+      <c r="F18" s="23">
+        <v>12</v>
+      </c>
+      <c r="G18" s="23">
+        <v>50</v>
+      </c>
+      <c r="H18" s="23">
+        <v>50</v>
+      </c>
+      <c r="I18" s="23">
+        <f>G18-H18</f>
+        <v>0</v>
+      </c>
+      <c r="J18" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="K18" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L18" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M18" s="22"/>
+      <c r="N18" s="22"/>
+      <c r="O18" s="22"/>
+      <c r="P18" s="22"/>
+      <c r="Q18" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>254</v>
+      </c>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22" t="s">
+        <v>255</v>
+      </c>
+      <c r="F19" s="23">
+        <v>1</v>
+      </c>
+      <c r="G19" s="23">
+        <v>0</v>
+      </c>
+      <c r="H19" s="23">
+        <v>25</v>
+      </c>
+      <c r="I19" s="23">
+        <f>-H19</f>
+        <v>-25</v>
+      </c>
+      <c r="J19" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="K19" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L19" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M19" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="N19" s="22"/>
+      <c r="O19" s="22"/>
+      <c r="P19" s="22"/>
+      <c r="Q19" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="22"/>
+      <c r="B20" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>256</v>
+      </c>
+      <c r="D20" s="22" t="s">
+        <v>257</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>258</v>
+      </c>
+      <c r="F20" s="23">
+        <v>11</v>
+      </c>
+      <c r="G20" s="23">
+        <v>615</v>
+      </c>
+      <c r="H20" s="23">
+        <v>25</v>
+      </c>
+      <c r="I20" s="23">
+        <f t="shared" ref="I20:I22" si="1">G20-H20</f>
+        <v>590</v>
+      </c>
+      <c r="J20" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="K20" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L20" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M20" s="22"/>
+      <c r="N20" s="22"/>
+      <c r="O20" s="22"/>
+      <c r="P20" s="22"/>
+      <c r="Q20" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="22"/>
+      <c r="B21" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>259</v>
+      </c>
+      <c r="D21" s="22" t="s">
+        <v>260</v>
+      </c>
+      <c r="E21" s="22" t="s">
+        <v>261</v>
+      </c>
+      <c r="F21" s="23">
+        <v>4</v>
+      </c>
+      <c r="G21" s="23">
+        <v>815</v>
+      </c>
+      <c r="H21" s="23">
+        <v>25</v>
+      </c>
+      <c r="I21" s="23">
+        <f t="shared" si="1"/>
+        <v>790</v>
+      </c>
+      <c r="J21" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="K21" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L21" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M21" s="22"/>
+      <c r="N21" s="22"/>
+      <c r="O21" s="22"/>
+      <c r="P21" s="22"/>
+      <c r="Q21" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="22"/>
+      <c r="B22" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" s="22" t="s">
+        <v>262</v>
+      </c>
+      <c r="D22" s="22" t="s">
+        <v>263</v>
+      </c>
+      <c r="E22" s="22" t="s">
+        <v>264</v>
+      </c>
+      <c r="F22" s="22" t="s">
+        <v>108</v>
+      </c>
+      <c r="G22" s="23">
+        <v>765</v>
+      </c>
+      <c r="H22" s="23">
+        <v>25</v>
+      </c>
+      <c r="I22" s="23">
+        <f t="shared" si="1"/>
+        <v>740</v>
+      </c>
+      <c r="J22" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="K22" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L22" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="M22" s="22"/>
+      <c r="N22" s="22"/>
+      <c r="O22" s="22"/>
+      <c r="P22" s="22"/>
+      <c r="Q22" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="G24" s="1">
+        <f>SUBTOTAL(9,G3:G23)</f>
+        <v>9860</v>
+      </c>
+      <c r="H24" s="1">
+        <f>SUBTOTAL(9,H3:H23)</f>
+        <v>580</v>
+      </c>
+      <c r="I24" s="1">
+        <f>SUBTOTAL(9,I3:I23)</f>
+        <v>9280</v>
+      </c>
+      <c r="J24" s="1">
+        <f>SUBTOTAL(9,J3:J23)</f>
+        <v>0</v>
+      </c>
+      <c r="K24" s="1">
+        <f>SUBTOTAL(9,K3:K23)</f>
+        <v>0</v>
+      </c>
+      <c r="L24" s="1">
+        <f>SUBTOTAL(9,L3:L23)</f>
+        <v>0</v>
+      </c>
+      <c r="M24" s="1">
+        <f>SUBTOTAL(9,M3:M23)</f>
+        <v>0</v>
+      </c>
+      <c r="N24" s="1">
+        <f>SUBTOTAL(9,N3:N23)</f>
+        <v>0</v>
+      </c>
+      <c r="O24" s="1">
+        <f>SUBTOTAL(9,O3:O23)</f>
+        <v>0</v>
+      </c>
+      <c r="P24" s="1">
+        <f>SUBTOTAL(9,P3:P23)</f>
+        <v>0</v>
+      </c>
+      <c r="Q24" s="1">
+        <f>SUBTOTAL(9,Q3:Q23)</f>
+        <v>20</v>
+      </c>
+      <c r="R24" s="1">
+        <f>SUBTOTAL(9,R3:R23)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="I25" s="1">
+        <v>-3055</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H28" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J28" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H29" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I29" s="8">
+        <f>SUM(I23:I27)</f>
+        <v>6225</v>
+      </c>
+      <c r="J29" s="8">
+        <f>Q24</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="H30" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="I30" s="10">
+        <f>R24</f>
+        <v>0</v>
+      </c>
+      <c r="J30" s="11"/>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="H31" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="I31" s="10">
+        <f>S23</f>
+        <v>0</v>
+      </c>
+      <c r="J31" s="11"/>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="H32" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="I32" s="10">
+        <f>T23</f>
+        <v>0</v>
+      </c>
+      <c r="J32" s="11"/>
+    </row>
+    <row r="33" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="H33" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="I33" s="10">
+        <f>U23</f>
+        <v>0</v>
+      </c>
+      <c r="J33" s="11"/>
+    </row>
+    <row r="34" spans="8:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H34" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="I34" s="13"/>
+      <c r="J34" s="13"/>
+    </row>
+    <row r="35" spans="8:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H35" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="I35" s="13"/>
+      <c r="J35" s="13"/>
+    </row>
+    <row r="36" spans="8:10" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="H36" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="I36" s="16">
+        <f>SUM(I29:I35)</f>
+        <v>6225</v>
+      </c>
+      <c r="J36" s="16">
+        <f>SUM(J29:J33)</f>
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:P22" xr:uid="{00000000-0009-0000-0000-000006000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:P22">
+      <sortCondition ref="J2:J22"/>
+    </sortState>
+  </autoFilter>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03AB5974-9CA3-40AA-9389-A33FB2F60527}">
   <dimension ref="A1:R70"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3838,10 +5151,10 @@
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>266</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>27</v>
+        <v>267</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
@@ -4994,7 +6307,7 @@
     </row>
     <row r="62" spans="1:18" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="H62" s="4" t="s">
-        <v>28</v>
+        <v>268</v>
       </c>
       <c r="I62" s="5" t="s">
         <v>15</v>

</xml_diff>